<commit_message>
Update zips and sample run with new changes.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/selections/Chain Ladder Selections - LDFs.xlsx
+++ b/sample-data/sample-run/selections/Chain Ladder Selections - LDFs.xlsx
@@ -4070,55 +4070,57 @@
     <row r="69">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Selection</t>
+          <t>Framework AI Selection</t>
         </is>
       </c>
       <c r="B69" s="18" t="n">
-        <v>1.68</v>
+        <v>1.7</v>
       </c>
       <c r="C69" s="18" t="n">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>1.165</v>
+        <v>1.125</v>
       </c>
       <c r="E69" s="18" t="n">
-        <v>1.049</v>
+        <v>1.037</v>
       </c>
       <c r="F69" s="18" t="n">
-        <v>1.09</v>
+        <v>1.105</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>1.075</v>
+        <v>1.087</v>
       </c>
       <c r="H69" s="18" t="n">
-        <v>1.0085</v>
+        <v>1.015</v>
       </c>
       <c r="I69" s="18" t="n">
-        <v>1.015</v>
+        <v>1.016</v>
       </c>
       <c r="J69" s="18" t="n">
-        <v>1.038</v>
+        <v>1.05</v>
       </c>
       <c r="K69" s="18" t="n">
-        <v>1.0075</v>
+        <v>1.002</v>
       </c>
       <c r="L69" s="18" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="M69" s="18" t="n">
-        <v>1.005</v>
+        <v>1.003</v>
       </c>
       <c r="N69" s="18" t="n">
-        <v>1.005</v>
+        <v>1.002</v>
       </c>
       <c r="O69" s="18" t="n">
         <v>1.01</v>
       </c>
       <c r="P69" s="18" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="Q69" s="19" t="n"/>
+        <v>1.005</v>
+      </c>
+      <c r="Q69" s="18" t="n">
+        <v>1.009</v>
+      </c>
       <c r="R69" s="19" t="n"/>
       <c r="S69" s="19" t="n"/>
       <c r="T69" s="19" t="n"/>
@@ -4130,90 +4132,94 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Reasoning</t>
+          <t>Framework AI Reasoning</t>
         </is>
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>1.6800 selected. High variance (CV_5yr=0.33, CV_3yr=0.16) with meaningful 3yr vs 5yr divergence (1.489 vs 1.702). The 3yr window is depressed by AY2020 (1.785) and AY2022 (1.226), while the 5yr picks up higher recent years (2018: 2.299, 2019: 2.757). Incurred severity is rising strongly in recent origin years (2022: ~2774 at age 35, 2023: ~5419 at age 23), and case reserves at age 11 are elevated and growing (2023: 607K, 2024: 535K), consistent with delayed case development requiring a higher factor. Paid-to-incurred ratios at 11 months are declining in recent years (2023: 0.38, 2024: 0.40), confirming large unreleased case reserves. No convergence — averages diverge over 14%. Asymmetric conservatism applied: movement upward from 5yr weighted (1.702) is credible given severity trend, but early maturity warrants Bayesian anchoring. Splitting the difference between 5yr VW and the 10yr VW (1.737), blending toward 1.68 acknowledges the recent severity signal while capping volatility at early maturity. All-weighted = 1.614 but this is dragged down by older low-severity AYs.</t>
+          <t>1.7000: cv_5yr=0.328 is very high (well above the 0.20 outlier-exclusion threshold), and the recency windows disagree in direction - weighted_3yr (1.4891) is actually below weighted_all (1.6135), while weighted_5yr (1.7024) and simple_5yr (1.784) sit well above it. This inconsistency is expected at the earliest, most volatile maturity (Section 9: outlier exclusion de-emphasized here). Selected close to the outlier-trimmed all-year average (avg_exclude_high_low_all=1.7265), balancing against the raw weighted_all figure. No prior exists, so no Bayesian anchoring was applied.</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
-          <t>1.2000 selected. CV_5yr=0.21 (high), CV_3yr=0.13. Recent AYs: 2020=0.983, 2021=1.224, 2022=0.972. The 3yr weighted (1.054) is heavily distorted by the two sub-1.0 factors (2020 and 2022), which are anomalous — sub-1.0 incurred LDFs at 23-35 months are possible (case reserve reductions) but require corroboration. The 5yr weighted (1.258) includes the strong 2018 and 2019 factors (1.429 and 1.547) and is more credible. Incurred severity progression confirms ongoing development in this range. The all-year weighted = 1.189 and 10yr = 1.288. Given the recent two-year depression in factors (potentially case reserve reductions in 2020 COVID period and 2022), treating these as partially transient and selecting near the midpoint of 5yr VW and all-year VW. Asymmetric conservatism applied (downward movement from 5yr, move 30-50% of gap): 5yr = 1.258, all = 1.189, gap from 5yr to selected = 0.058. Selection of 1.200 reflects modest conservatism, staying above the anomalous 3yr average.</t>
+          <t>1.2200: cv_5yr=0.21 exceeds the outlier-exclusion threshold. weighted_3yr (1.054) is pulled down by two recent diagonals near or below 1.0 (2022=0.9715, 2020=0.9832), which is unusual for incurred development this early and would require diagnostic confirmation of decreasing case reserve adequacy before being trusted at full weight - that confirmation is not clearly present. Selected near the outlier-trimmed 5-year average (avg_exclude_high_low_5yr=1.212), rejecting the low 3-year figure per Section 11 (incurred LDFs should not select below 1.000, and the raw 3yr average is too close to that floor to be reliable).</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>1.1650 selected. CV_5yr=0.13, CV_3yr=0.057 (low-moderate). 3yr VW=1.095, 5yr VW=1.200, 10yr VW=1.189, all VW=1.153. Recent AYs trend lower: 2020=1.058, 2021=1.032, 2022 has no 35-47 factor yet. The 3yr is materially below the 5yr (gap ~10.5%). Incurred severity shows heterogeneous development in this range — some AYs resolve quickly, others don't. Applying partial convergence weighting: 5yr VW (1.200) has meaningful CV suggesting more weight on 5yr vs 3yr. Mid-maturity range, relaxed asymmetric conservatism. Selected as blend: 60% on 5yr (1.200) + 40% on 3yr (1.095) = ~1.158, rounded up slightly to 1.165 for conservative bias at this still-early maturity stage.</t>
+          <t>1.1250: weighted_3yr (1.0948) is 8.8% below weighted_5yr (1.2002), exceeding the &gt;5% divergence threshold, driven by a genuine multi-year decline (2019=1.15, 2020=1.058, 2021=1.03) versus older, higher years (2015=1.33, 2018=1.39) - consistent with faster claims resolution over time. Weighted roughly 70% toward the 3-year figure and 30% toward the 5-year figure (1.0948*0.7+1.2002*0.3=1.1265), rounded to 1.1250, since diagnostic support is only indirect (not a full 75-100% shift).</t>
         </is>
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>1.0490 selected. CV_5yr=0.056, CV_3yr=0.036 (both low). All averages converge well: 3yr VW=1.023, 5yr VW=1.057, 10yr VW=1.057, all VW=1.049. The 3yr appears slightly low (1.023) due to AY2020 (1.010), otherwise factors are stable in the 1.04-1.14 range for most AYs. Partial convergence between 5yr and all-year (within ~1%). 5yr VW of 1.057 is consistent with all-year. Selection of 1.049 follows the volume-weighted all-year average which best captures the central tendency in a stable column with moderate data.</t>
+          <t>1.0370: weighted_3yr (1.0233) vs weighted_5yr (1.0567) diverge 3.16%, in the 3-5% band. Blended 60% 5yr / 40% 3yr per Section 6 (0.6*1.0567+0.4*1.0233=1.0367), rounded to 1.0370.</t>
         </is>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
-          <t>1.0900 selected. CV_5yr=0.077, CV_3yr=0.093 (moderate). 3yr VW=1.117, 5yr VW=1.103, 10yr VW=1.075, all VW=1.074. Recent trend is slightly upward — 2019=1.222, 2020=1.010, while 2017=1.133 and 2018=1.013. The 3yr and 5yr are elevated relative to all-year, indicating recent LDFs are running higher. The slope over 3yr is positive (0.045). However, the 2019 factor (1.222) is the highest recent point, and 2020 (1.010) follows up as a potentially COVID-affected low. Incurred severity in recent AYs for this maturity range is elevated. Select near the 5yr VW (1.103), dampened slightly toward the all-year (1.074), reflecting trending but with asymmetric conservatism on the upside movement. Selection of 1.090 represents approximately 60% weight on the 5yr VW.</t>
+          <t>1.1050: weighted_3yr (1.1167) and weighted_5yr (1.1027) closely agree (1.25% apart) and both exceed the all-year average (1.0736) by ~3%, mirroring the same rise observed in the Paid Loss triangle at this interval - cross-view (paid/incurred) correlation supports treating this as a real, moderate upward move. Selected near weighted_5yr.</t>
         </is>
       </c>
       <c r="G70" s="20" t="inlineStr">
         <is>
-          <t>1.0750 selected. CV_5yr=0.074, CV_3yr=0.061. 3yr VW=1.090, 5yr VW=1.087, 10yr VW=1.067, all VW=1.046. The 3yr and 5yr averages are consistent with each other and notably above the 10yr/all-year, indicating a regime shift toward higher development in recent years. Incurred severity data supports ongoing case reserve increases. Paid-to-incurred ratios in mid-maturity remain below benchmark in recent AYs (e.g., 2017: 0.844, 2018: 0.969, 2019: 0.921), suggesting case reserves remain active. 3yr slope is positive at 0.45 but recent 2 LDFs (2018: 1.027, 2019: not yet visible at 71-83) show some stabilization. Selection of 1.075 is approximately equal to the 5yr VW, supported by convergence of 3yr and 5yr, with slight dampening from 10yr.</t>
+          <t>1.0870: This is a late-maturity column, but weighted_3yr (1.0898) and weighted_5yr (1.087) agree tightly and both sit ~4% above weighted_all (1.0457) - and this matches the analogous Paid Loss selection at 71-83 (1.088), giving cross-view confirmation of a genuine, ongoing severity trend rather than noise. Selected the 5-year weighted average.</t>
         </is>
       </c>
       <c r="H70" s="20" t="inlineStr">
         <is>
-          <t>1.0085 selected. CV_5yr=0.014 (low), CV_3yr=0.016. Very stable column. 3yr VW=1.009, 5yr VW=1.007, 10yr VW=1.018, all VW=1.022. Recent LDFs are low: 2017=1.032, 2016=1.000, 2018=N/A at this maturity. The convergence between 3yr and 5yr VW (within 0.2%) is strong. All-year is slightly higher due to older AYs. Selection follows 5yr VW closely. No trend signal, low CV — stable development at this maturity.</t>
+          <t>1.0150: Low variance (cv_3yr=0.016, cv_5yr=0.014). weighted_all (1.0221) sits modestly above the recency windows (1.0065-1.0085); per late-maturity guidance (prefer all-year absent a structural break), selected a blend closer to the midpoint.</t>
         </is>
       </c>
       <c r="I70" s="20" t="inlineStr">
         <is>
-          <t>1.0150 selected. CV_5yr=0.025, CV_3yr=0.022 (low). 3yr VW=1.010, 5yr VW=1.013, 10yr VW=1.023, all VW=1.020. Recent factors are low (2016: 1.001, 2015: 1.003) while older AYs (2007: 1.072) pull up the all-year. The 5yr and 3yr averages converge around 1.010-1.015. Selection at 1.015 is slightly above the 5yr VW to account for the possibility that recent very-low factors in 2015-2016 understate long-run development, consistent with the 10yr average of 1.023. Incurred severity at this maturity shows ongoing small increases in some AYs.</t>
+          <t>1.0160: weighted_all (1.0195), weighted_5yr (1.0146), weighted_3yr (1.0098) are closely converged (within ~1%). Selected the midpoint.</t>
         </is>
       </c>
       <c r="J70" s="20" t="inlineStr">
         <is>
-          <t>1.0380 selected. CV_5yr=0.039, CV_3yr=0.049 (low-moderate). 3yr VW=1.063, 5yr VW=1.049, 10yr VW=1.052, all VW=1.037. Recent factors include 2015: 1.096 (notably high, driven by case reserve increases visible in the 2015 case reserve data). 2016: N/A, 2014: 1.021. The 3yr is elevated due to 2015's 1.096 factor. The 5yr and 10yr converge around 1.049-1.052 and are most credible. Selection of 1.038 follows the all-year weighted which best reflects central tendency excluding the 2015 outlier influence, consistent with stable mid-late development.</t>
+          <t>1.0500: weighted_5yr (1.0485) is modestly above weighted_all (1.037), a mild uptick that is consistent (not diverging materially, 1.4%) between the 3-year (1.0629) and 5-year windows. Selected near the 5-year weighted average.</t>
         </is>
       </c>
       <c r="K70" s="20" t="inlineStr">
         <is>
-          <t>1.0075 selected. CV_5yr=0.013, CV_3yr=0.007 (very low). All averages converge tightly: 3yr VW=1.000, 5yr VW=1.008, 10yr VW=1.019, all VW=1.017. The 3yr is pinned to 1.000 by three consecutive 1.000 factors for AYs 2013-2015. The 5yr and 10yr are slightly higher. Convergence override does not fully apply since 3yr vs 5yr diverge by ~0.8pp. Selection at 1.0075, midpoint of the 3yr (1.000) and 5yr (1.008), reflecting the stable low-development pattern at this late maturity.</t>
+          <t>1.0020: weighted_3yr (0.9997) is essentially at unity with very low cv_3yr (0.007), and avg_exclude_high_low_5yr (1.0028) confirms a similar level. Per Section 11 (late maturity, incurred can go as low as 0.995-1.000 with multi-year confirmation), the low, consistent multi-year reading supports a selection at/just above 1.000 rather than defaulting higher; selected 1.0020 to stay safely at or above unity.</t>
         </is>
       </c>
       <c r="L70" s="20" t="inlineStr">
         <is>
-          <t>1.0300 selected. CV_5yr=0.076, CV_3yr=0.099 (moderate). 3yr VW=1.053, 5yr VW=1.035, 10yr VW=1.040, all VW=1.033. The high CV is driven by AY2012 (1.179), which is a clear outlier (large reserve strengthening in one period). Excluding the outlier, 5yr ex-hi/lo = 1.005 which goes too far down. The all-year VW (1.033) and 5yr VW (1.035) converge nicely and represent credible central tendency. Selection follows 5yr/all-year convergence, reflecting normal case reserve fluctuation at this mature age.</t>
+          <t>1.0100: cv_3yr=0.099 is near the 0.10 outlier-exclusion threshold, and avg_exclude_high_low_5yr (1.0045) is materially lower than the raw weighted_5yr (1.035), indicating a single elevated diagonal (2012=1.179) is inflating the untrimmed averages. Selected close to the outlier-trimmed figure.</t>
         </is>
       </c>
       <c r="M70" s="20" t="inlineStr">
         <is>
-          <t>1.0050 selected. CV_5yr=0.016 (very low). All averages converge: 3yr=1.000, 5yr VW=1.002, 10yr VW=1.007, all VW=1.005. Near-convergence across all windows (within 0.7pp). 5yr VW and all VW are essentially identical. Selection follows the all-year VW of 1.005, reflecting very small residual development at this maturity. Late maturity behavior consistent.</t>
+          <t>1.0030: Very low variance (cv_3yr=0.0008); weighted_all (1.0053), weighted_5yr (1.0022), weighted_3yr (1.0004) are tightly converged. Selected the midpoint.</t>
         </is>
       </c>
       <c r="N70" s="20" t="inlineStr">
         <is>
-          <t>1.0050 selected. CV very low (3yr=0.000, 5yr=0.000). All averages essentially converge: 3yr=1.000, 5yr=1.000, all VW=1.005, 10yr=1.003. The all-year VW pulls slightly above 1.000 due to AY2001 (1.023) and AY2002 (1.040). Selection of 1.005 follows the all-year VW, which captures the full history of residual development at this late maturity stage.</t>
+          <t>1.0020: Convergence Override - cv_3yr=0.0001 and cv_5yr=0.0004 indicate near-total agreement across all averaging windows (weighted_all=1.0054, weighted_5yr=1.0004, weighted_3yr=0.9999). Selected the midpoint of the converged band.</t>
         </is>
       </c>
       <c r="O70" s="20" t="inlineStr">
         <is>
-          <t>1.0100 selected. CV low (3yr=0.004, 5yr=0.019). 3yr=1.002, 5yr VW=1.021, 10yr VW=1.017, all VW=1.017. Some variation across windows. At late maturity (167+ months), all-year window appropriate per guidelines. All-year VW of 1.017 and 10yr VW of 1.017 converge. Selection of 1.010 applies modest conservatism below the all-year (some recent AYs showing zero development confirms declining tail).</t>
+          <t>1.0100: weighted_3yr (1.002) sits below weighted_5yr (1.0211) and weighted_all (1.0167), reflecting a mild recent stabilization at this depth. Selected a blended value between the recent and longer-term figures.</t>
         </is>
       </c>
       <c r="P70" s="20" t="inlineStr">
         <is>
-          <t>CUTOFF at 179 months: This is the last selected interval before the tail begins. CV is very low (5yr=0.005, 3yr=0.003). Averages: 3yr=1.001, 5yr VW=1.004, 10yr VW=1.012, all VW=1.012. Most recent AYs showing 1.000-1.005 range. Selection of 1.003 reflects the low recent development visible in the 3yr and 5yr averages, consistent with declining tail activity. The pattern at 179+ months is monotonically very small and converging to 1.000.</t>
+          <t>1.0050: Low variance (cv_3yr=0.003, cv_5yr=0.005); weighted_all (1.0116), weighted_5yr (1.0036), weighted_3yr (1.0009) converge toward a flat, near-unity pattern typical of this maturity. Selected between the recent and all-year figures.</t>
         </is>
       </c>
       <c r="Q70" s="20" t="inlineStr">
         <is>
-          <t>[CUTOFF] CUTOFF at 191 months: is_monotone_from_here=True, CV at this interval is near-zero (3yr=0.010, 5yr=0.009), factors are stable near 1.005-1.015 range but sparse. Only a few points remain in each column at this maturity, satisfying sparse data caution. Rejected further selection (191+) due to fewer than 5 credible data points per interval and near-zero incremental development. Tail curve fitting should commence from 191 months using the residual CDF. Minimum cutoff for Incurred Loss (48 months) is exceeded.</t>
-        </is>
-      </c>
-      <c r="R70" s="8" t="n"/>
+          <t>1.0090: weighted_all (1.0149), weighted_5yr (1.0076), weighted_3yr (1.0066) are closely aligned; selected between the all-year and recency-weighted figures. This is the last interval selected before the tail cutoff - cv_5yr=0.0089, low and stable, giving a credible endpoint for observed development consistent with the Paid Loss cutoff at the same age for internal consistency.</t>
+        </is>
+      </c>
+      <c r="R70" s="20" t="inlineStr">
+        <is>
+          <t>[CUTOFF] CUTOFF at 215 months (well beyond the 48-month Incurred Loss minimum). Beyond this point, cv_5yr values stay very low (0.0-0.0188) and factors sit in a tight band around 1.0 (0.9938-1.0174) with only noise-level slope changes rather than a structural break. 7 intervals remain (203-215 through 275-287) for tail curve fitting, comfortably meeting the ≥3-5 requirement, and the cutoff aligns with the Paid Loss cutoff at the same maturity for internal consistency between the two loss triangles. The final column (275-287) has only a single accident-year observation, confirming this region is better extrapolated via curve fit than hand-selected.</t>
+        </is>
+      </c>
       <c r="S70" s="8" t="n"/>
       <c r="T70" s="8" t="n"/>
       <c r="U70" s="8" t="n"/>
@@ -4229,37 +4235,37 @@
         </is>
       </c>
       <c r="B72" s="22" t="n">
-        <v>1.7</v>
+        <v>1.75</v>
       </c>
       <c r="C72" s="22" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="D72" s="22" t="n">
-        <v>1.12</v>
+        <v>1.15</v>
       </c>
       <c r="E72" s="22" t="n">
-        <v>1.05</v>
+        <v>1.048</v>
       </c>
       <c r="F72" s="22" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="G72" s="22" t="n">
-        <v>1.06</v>
+        <v>1.065</v>
       </c>
       <c r="H72" s="22" t="n">
-        <v>1.02</v>
+        <v>1.015</v>
       </c>
       <c r="I72" s="22" t="n">
-        <v>1.02</v>
+        <v>1.017</v>
       </c>
       <c r="J72" s="22" t="n">
-        <v>1.035</v>
+        <v>1.048</v>
       </c>
       <c r="K72" s="22" t="n">
-        <v>1.015</v>
+        <v>1.012</v>
       </c>
       <c r="L72" s="22" t="n">
-        <v>1.03</v>
+        <v>1.028</v>
       </c>
       <c r="M72" s="22" t="n">
         <v>1.005</v>
@@ -4271,25 +4277,25 @@
         <v>1.01</v>
       </c>
       <c r="P72" s="22" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="Q72" s="22" t="n">
-        <v>1.01</v>
+        <v>1.011</v>
       </c>
       <c r="R72" s="22" t="n">
-        <v>1.005</v>
+        <v>1.006</v>
       </c>
       <c r="S72" s="22" t="n">
         <v>1.003</v>
       </c>
       <c r="T72" s="22" t="n">
-        <v>1.005</v>
+        <v>1.004</v>
       </c>
       <c r="U72" s="22" t="n">
-        <v>1.005</v>
+        <v>1.004</v>
       </c>
       <c r="V72" s="22" t="n">
-        <v>1.015</v>
+        <v>1.014</v>
       </c>
       <c r="W72" s="22" t="n">
         <v>1</v>
@@ -4304,117 +4310,117 @@
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>1.7000. The all-period weighted average is 1.614 and simple average is 1.744. The 3-year average (1.489) reflects a recent dip but the 5-year (1.784) and 10-year (1.774) simple averages support higher values. The data is highly variable (CV_10yr = 0.269) with individual factors ranging from 1.089 to 2.757. Recent years 2019-2023 show elevated factors (2.757, 1.785, 1.458, 1.226, 1.694), suggesting the book has periods of very high early reporting. The 3-year low reflects 2022 (1.226) and 2021 (1.458) which appear to be low outlier years relative to the broader pattern. A selection of 1.70 is modestly below the simple-all average of 1.74 but above the weighted-all of 1.61, reflecting the high dispersion and the tendency for older years to have more low factors that pull down the weighted average.</t>
+          <t>1.75 selected. This is the largest and most volatile link (cv_3yr 0.16, cv_5yr 0.33) reflecting the initial incurred build-up as claims are first reported and reserved. Individual factors range widely (1.09 in 2007 to 2.76 in 2019) with no clear trend, so the selection anchors near simple_all (1.7435) and weighted_10yr (1.7371) rather than the noisier 3-year window (1.4891), which is skewed low by 2020-2022.</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>1.2000. The weighted-all average is 1.189 and simple-all is 1.193. The 3-year simple average is 1.060 and 5-year is 1.231. The 10-year averages cluster around 1.25-1.29. Recent years show very low factors: 2022 (0.9715), 2021 (1.224), 2020 (0.983), 2023 (N/A). The 2022 factor below 1.0 is unusual and likely reflects timing. The 2006 factor of 0.869 also shows downward outliers. Most middle-period years show factors in 1.05-1.50 range. A selection of 1.20 is near the weighted-all average, acknowledging that the recent low 3-year period may be anomalous while the overall pattern centers around 1.19-1.19. The 10-year weighted average of 1.288 would also be defensible, but 1.20 appropriately weights recent experience.</t>
+          <t>1.15 selected. Averages diverge by window (weighted_all 1.1891, 3yr 1.054, 5yr 1.2575, 10yr 1.2877); the most recent 3 years (2020-2022: 0.9832, 1.224, 0.9715) run notably lower than history. Selection splits between the recent softening and the longer-term level, favoring a modest reduction from the all-year average.</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>1.1200. Weighted-all is 1.153, simple-all is 1.154. The 3-year average is 1.080 and 5-year is 1.187. The 10-year averages are around 1.181-1.188. Recent years are more moderate: 2021 (1.032), 2020 (1.058), 2022 (N/A). The 2008 factor of 1.391 and 2018 (1.388) are high outliers. Excluding those, the central tendency is in the 1.07-1.16 range. A selection of 1.12 is slightly below the all-period averages but reflects the modest downward drift in recent years and the concentration of factors in a credible range.</t>
+          <t>1.15 selected, between weighted_all (1.153) and the lower recent 3yr figure (1.0948), which reflects softer development in 2021-2022. Longer windows (5yr 1.2002, 10yr 1.1886) argue for keeping the selection above the 3yr trough.</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>1.0500. The weighted-all is 1.049 and simple-all is 1.049. The 3-year average is 1.023, 5-year is 1.057. Most years cluster tightly in the 1.00-1.08 range, with 2003 (0.908) and 2005 (0.975) as low outliers from early years. Recent factors are 1.010 (2020), 1.063 (2019). The CV drops to 0.047-0.056, indicating reasonable stability. A selection of 1.050 aligns well with both the weighted-all and simple-all averages, consistent across multiple time windows.</t>
+          <t>1.048 selected, consistent with weighted_all (1.0492), 5yr (1.0567) and 10yr (1.0574); the 3yr figure (1.0233) is a bit lower but the difference is small and within normal noise.</t>
         </is>
       </c>
       <c r="F73" s="24" t="inlineStr">
         <is>
-          <t>1.0800. This interval shows notable volatility with a wide range (0.989-1.222) and a 5yr CV of 0.077. The 3-year average (1.117) is elevated relative to the longer-term averages (weighted-all 1.074, simple-all 1.062). Recent years show higher development: 2019 (1.222), 2018 (1.013), 2017 (1.133), reflecting an upward shift in this interval in recent years. The 2007 year had a very high factor of 1.194 that contributed to long-run averages. The slope shows a modest upward trend in the 3-year window. A selection of 1.080 is above the longer-term weighted-all (1.074) but below the 3-year average, giving credit to the recent elevated pattern while acknowledging some regression to the mean.</t>
+          <t>1.09 selected, close to weighted_all (1.0736) but reflecting the somewhat elevated recent windows (3yr 1.1167, 5yr 1.1027, 10yr 1.0752), consistent with slightly more late incurred development in the most recent cohorts.</t>
         </is>
       </c>
       <c r="G73" s="24" t="inlineStr">
         <is>
-          <t>1.0600. The weighted-all is 1.046, simple-all is 1.040, but the 3-year average is 1.090 and the 5-year average is 1.087. Recent years (2019: N/A, 2018: 1.027, 2017: 1.153, 2016: 1.128, 2015: 1.140) show a distinct upward shift since 2015, with several years in the 1.10-1.15 range — well above the historical average. This recent severity increase appears genuine and driven by the same pattern seen at earlier ages. The 5-year weighted average of 1.087 and the 3-year of 1.090 dominate here. A selection of 1.060 balances the longer-term pattern against recent emergence, falling between the long-run average and recent elevated experience.</t>
+          <t>1.065 selected, near the consensus of 5yr (1.087) and 10yr (1.0671) averages, moderated from the highest recent 3yr figure (1.0898) which is influenced by a couple of larger factors (2017: 1.1527).</t>
         </is>
       </c>
       <c r="H73" s="24" t="inlineStr">
         <is>
-          <t>1.0200. The weighted-all is 1.022, simple-all is 1.021. The 3-year average is 1.013 and 5-year is 1.008. CV is low (0.016-0.044). Most factors are in a tight 1.00-1.05 range, with 2009 (1.144) as a notable outlier driven by a reserve strengthening event. Excluding the 2009 outlier, the remaining factors are 0.98-1.11. The all-period average captures this well. A selection of 1.020 is consistent with the weighted-all and recognizes this interval has modest but real residual development.</t>
+          <t>1.015 selected, between weighted_all (1.0221) and the lower recent windows (3yr 1.0085, 5yr 1.0065), reflecting continued but diminishing development as claims mature toward settlement.</t>
         </is>
       </c>
       <c r="I73" s="24" t="inlineStr">
         <is>
-          <t>1.0200. The weighted-all is 1.020, simple-all is 1.018. The 3-year average is 1.010 and 5-year is 1.015. CV is low (0.022-0.027). Factors range from 0.995 to 1.072. The weighted average across all years (1.020) is the most credible anchor here. Selected at 1.020 consistent with all-period weighted average and stable pattern.</t>
+          <t>1.017 selected, close to weighted_all (1.0195) and 10yr (1.0231), slightly favoring the somewhat lower recent windows (3yr 1.0098, 5yr 1.0146).</t>
         </is>
       </c>
       <c r="J73" s="24" t="inlineStr">
         <is>
-          <t>1.0350. The weighted-all is 1.037, simple-all is 1.026. The 5-year average is 1.049 and 10-year weighted is 1.052. Notable outlier is 2007 (1.102) — a large loss year driving the weighted average up. Recent years: 2015 (1.096), 2016 (N/A). The 3-year simple average is 1.039. Data becomes sparse at this age. Selecting 1.035 is between the simple-all and weighted-all, acknowledging some positive development in this interval historically, noting the 2007 outlier effect on the weighted average.</t>
+          <t>1.048 selected, aligned with weighted_all (1.037) through 10yr (1.0519) and the elevated 3yr figure (1.0629). This interval carries genuine incremental development from case reserve strengthening in a few years (e.g., 2015: 1.0962, 2012: 1.0565), so the selection stays near the higher end of the observed range rather than dampening toward the long-run mean alone.</t>
         </is>
       </c>
       <c r="K73" s="24" t="inlineStr">
         <is>
-          <t>1.0150. The weighted-all is 1.017, simple-all is 1.015. The 3-year average is essentially 1.000, 5-year is 1.008. CV is low (0.007-0.026). Most factors are very close to 1.000-1.010, with 2006 (1.083) and 2007 (1.031) as higher outliers from specialty years. Recent experience suggests factors near 1.0. A selection of 1.015 gives modest credit for the historical positive development pattern while reflecting recent near-flat experience.</t>
+          <t>1.012 selected, between weighted_all (1.0174) and the near-flat recent 3yr figure (0.9997), which reflects a run of years with little to no late development at this maturity.</t>
         </is>
       </c>
       <c r="L73" s="24" t="inlineStr">
         <is>
-          <t>1.0300. The weighted-all is 1.033, simple-all is 1.033, but with notable dispersion (CV ~0.07-0.10). The 5-year average is 1.038 and 3-year is 1.053. The 2012 factor (1.179) is a large outlier. Recent years 2011 (0.997), 2010 (0.000 flagged), 2009 (1.014) show variability. The weighted average is pulled up by 2005 (1.119) and 2012 (1.179). A selection of 1.030 is near the all-period averages, representing reasonable development at this age.</t>
+          <t>1.028 selected. The weighted_all (1.0332) and 10yr (1.0395) figures are inflated by a single large outlier (2012: 1.179); avg_exclude_high_low_all (1.0242) strips that out and is closer to the true central tendency. Selection sits between the trimmed average and the raw weighted average to retain some allowance for the observed reserve-strengthening event.</t>
         </is>
       </c>
       <c r="M73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. The weighted-all is 1.005, simple-all is 1.005. CV is very low (0.001-0.016). Factors cluster tightly around 1.000-1.030. The 2009 factor (1.030) is highest. Recent years show nearly 1.000. A selection of 1.005 aligns with the central tendency.</t>
+          <t>1.005 selected, matching weighted_all (1.0053) and the trimmed average (1.004) closely; a low-volatility, well-developed interval.</t>
         </is>
       </c>
       <c r="N73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. The weighted-all is 1.005, simple-all is 1.005. Very stable — most factors within 1.000-1.040. CV is 0.001-0.015. A selection of 1.005 is appropriate.</t>
+          <t>1.005 selected, consistent with weighted_all (1.0054) and 10yr (1.003). Minor, stable residual incurred development.</t>
         </is>
       </c>
       <c r="O73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.017, simple-all is 1.010. The 5-year average is 1.021. Some residual development persists — 2001 (1.017), 2002 (1.026), 2007 (1.044). CV is moderate (0.015-0.019). A selection of 1.010 reflects the simple-all average, appropriate for this age.</t>
+          <t>1.010 selected. Weighted_all (1.0167) is pulled up by a single large 2001 factor (1.0532); avg_exclude_high_low_all (1.0075) removes that influence. Selection lands between the two, giving partial credit to the outlier without fully adopting it.</t>
         </is>
       </c>
       <c r="P73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all and simple-all both show 1.011-1.012. The 5-year average is 1.004. Factors range 1.000-1.053, with 2001 (1.053) as an outlier. Most years are at or near 1.000. A selection of 1.010 is consistent with the historical average.</t>
+          <t>1.009 selected, between weighted_all (1.0116) and the trimmed average (1.006), reflecting generally low, consistent late development at this maturity.</t>
         </is>
       </c>
       <c r="Q73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.015, simple-all is 1.015. The 3-year average is 1.007 and 5-year is 1.008. Factors range 1.000-1.053. A selection of 1.010 reflects the pattern with modest positive development at this age.</t>
+          <t>1.011 selected, between weighted_all (1.0149) and the trimmed/recent windows (avg_exclude_hl 1.0114, 3yr 1.0066), balancing a couple of larger observed factors against an otherwise flat pattern.</t>
         </is>
       </c>
       <c r="R73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. Weighted-all and simple-all are both around 1.006-1.007. Recent 3-year and 5-year averages are 1.002-1.003. Very stable with nearly all factors at 1.000. A selection of 1.005 captures residual development.</t>
+          <t>1.006 selected, matching weighted_all (1.0069) and 10yr (1.0069) closely, consistent with continued minor development.</t>
         </is>
       </c>
       <c r="S73" s="24" t="inlineStr">
         <is>
-          <t>1.0030. All averages show 1.003-1.005. Nearly all individual factors are 1.000. The simple/weighted averages across all periods are 1.003-1.005. Selected at 1.003.</t>
+          <t>1.003 selected. Weighted_all (1.0045) reflects one modest outlier against several years at 1.0; avg_exclude_high_low_all is exactly 1.0. Selection is set slightly above unity to retain a small allowance for residual movement.</t>
         </is>
       </c>
       <c r="T73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. Weighted-all is 1.009, simple-all is 1.009. The 3-year averages are 1.000. Several years show 1.000 and a few show 1.042 (2002). The weighted average gives more weight to larger observations. A conservative selection of 1.005 reflects modest development.</t>
+          <t>1.004 selected. Similar pattern to the prior interval — weighted_all (1.0089) is driven by one year (2007: 1.0424) against a mostly flat pattern (avg_exclude_high_low_all 1.0). A small positive factor is retained given the observed variability of loss development at very late durations.</t>
         </is>
       </c>
       <c r="U73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. Weighted-all is 1.007, simple-all is 1.004. Some factors at 1.000 and some at 1.023 (2001). A selection of 1.005 is consistent.</t>
+          <t>1.004 selected, similar rationale to the prior interval — weighted_all (1.0069) reflects one elevated factor against an otherwise flat pattern (avg_exclude_high_low_all 1.0).</t>
         </is>
       </c>
       <c r="V73" s="24" t="inlineStr">
         <is>
-          <t>1.0150. The weighted-all and simple-all are both 1.017. The only observation is 2001 (1.014) and 2002 (1.036). With limited data at this age, 1.015 is reasonable, reflecting the central tendency of available factors.</t>
+          <t>1.014 selected, matching weighted_all (1.0174) and avg_exclude_high_low_all (1.0139) reasonably closely; this interval shows more consistent development across the (few) mature origin years than the immediately preceding intervals.</t>
         </is>
       </c>
       <c r="W73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. All averages show 1.000. Both available years (2001, 2002) show 1.000. Selected at 1.000.</t>
+          <t>1.000 selected. Both available origin years at this maturity (2001 and 2002) show exactly 1.0, indicating claims are fully settled/incurred by this point for this book. This is the last interval selected directly from data with at least two corroborating observations.</t>
         </is>
       </c>
       <c r="X73" s="24" t="inlineStr">
         <is>
-          <t>[CUTOFF] Cutoff at 275 months. Only one observation available (2001: 1.012). With a single data point at this age, the tail curve fitting is more appropriate than a direct LDF selection. Development beyond 275 months is sparse and a tail factor from an actuarial tail curve (e.g., inverse power or exponential) should be applied from 275 months to ultimate.</t>
+          <t>[CUTOFF] Cutoff at 287: only a single origin year (2001) has data at this maturity (factor 1.0119), which is insufficient to validate a standalone selection. A fitted tail curve is more appropriate than extrapolating a one-point observation for the remaining runout.</t>
         </is>
       </c>
     </row>
@@ -8001,55 +8007,57 @@
     <row r="69">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Selection</t>
+          <t>Framework AI Selection</t>
         </is>
       </c>
       <c r="B69" s="18" t="n">
-        <v>2.55</v>
+        <v>2.5525</v>
       </c>
       <c r="C69" s="18" t="n">
-        <v>1.38</v>
+        <v>1.34</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>1.18</v>
+        <v>1.145</v>
       </c>
       <c r="E69" s="18" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="F69" s="18" t="n">
-        <v>1.11</v>
+        <v>1.125</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>1.115</v>
+        <v>1.088</v>
       </c>
       <c r="H69" s="18" t="n">
-        <v>1.03</v>
+        <v>1.029</v>
       </c>
       <c r="I69" s="18" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="J69" s="18" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="K69" s="18" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="L69" s="18" t="n">
+        <v>1.021</v>
+      </c>
+      <c r="M69" s="18" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="N69" s="18" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="O69" s="18" t="n">
+        <v>1.009</v>
+      </c>
+      <c r="P69" s="18" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="Q69" s="18" t="n">
         <v>1.013</v>
       </c>
-      <c r="J69" s="18" t="n">
-        <v>1.055</v>
-      </c>
-      <c r="K69" s="18" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L69" s="18" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="M69" s="18" t="n">
-        <v>1.015</v>
-      </c>
-      <c r="N69" s="18" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="O69" s="18" t="n">
-        <v>1.0075</v>
-      </c>
-      <c r="P69" s="18" t="n">
-        <v>1.0025</v>
-      </c>
-      <c r="Q69" s="19" t="n"/>
       <c r="R69" s="19" t="n"/>
       <c r="S69" s="19" t="n"/>
       <c r="T69" s="19" t="n"/>
@@ -8061,90 +8069,94 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Reasoning</t>
+          <t>Framework AI Reasoning</t>
         </is>
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>2.5500 selected. High variance (CV_5yr=0.18, CV_3yr=0.25), 24 data points. 3yr VW=2.629, 5yr VW=2.623, 10yr VW=2.482, all VW=2.457. Notably, 3yr and 5yr VW are nearly identical (within 0.3%), providing a strong convergence signal at the recent range. This near-convergence at the 3yr/5yr level takes priority over the lower all-year average (which is pulled down by older, lower-severity AYs from 2007-2013). Recent AYs: 2022=2.429, 2021=1.998, 2020=2.554, 2019=2.675, 2018=2.875. Incurred severity trending strongly upward in the 2022-2024 period (age-11 severity: 2022=2659, 2023=3569, 2024=3477), supporting elevated early-age paid LDFs. Paid-to-incurred at age 11 is low and declining (2023: 0.377, 2024: 0.399), indicating large remaining case reserves and substantial future paid development. 3yr/5yr convergence override applies: midpoint ~2.626 selected, then modest Asymmetric Conservatism applied (AY2021's 1.998 is an outlier pulling 3yr down slightly). Selection of 2.550 represents the convergence midpoint dampened by ~3% to account for the variance in the recent window and one potentially anomalous low point (2021=1.998).</t>
+          <t>2.5525: cv_5yr=0.177 falls in the 0.10-0.20 band, so the single highest and lowest 5-year LDFs were excluded (avg_exclude_high_low_5yr=2.5525) rather than using the raw weighted average. Early-maturity variance is naturally high (Section 9) so outlier exclusion is applied lightly. 3yr (2.6286) and 5yr (2.6232) weighted averages agree closely and both sit above the all-year average (2.4566), consistent with a genuine upward trend in early paid development corroborated by rising paid_severity_incr in recent accident years (e.g. 2016-2019 severities several times the 2001-2010 level). No prior selection exists so no Bayesian anchoring was applied.</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
-          <t>1.3800 selected. CV_5yr=0.21, CV_3yr=0.25 (high). 3yr VW=1.267, 5yr VW=1.422, 10yr VW=1.391, all VW=1.344. Wide divergence between 3yr and 5yr (&gt;15%). Recent AYs: 2020=1.180, 2021=1.666, 2022=1.060. AY2022 (1.060) and AY2020 (1.180) are anomalously low, pulling the 3yr average down. AY2019 (1.750) is the highest recent observation and may represent a large-loss AY. Incurred severity at age 23 rising sharply (2023: 5419). The 5yr and 10yr averages (1.422 and 1.391) are more credible than the 3yr. CV&gt;0.20 triggers outlier exclusion: the 5yr ex-hi/lo = 1.444. With the recent 3yr average suppressed by COVID-era and post-COVID anomalies, and the 5yr/10yr converging near 1.39-1.44, select near 1.380. This is the midpoint between 10yr VW (1.391) and all VW (1.344), reflecting a modest downward adjustment from the 5yr for the spike in 2019 while staying well above the 3yr anomaly.</t>
+          <t>1.3400: cv_5yr=0.21 (&gt;0.20) with 3yr and 5yr weighted averages diverging sharply (1.2671 vs 1.4224) driven by a single low recent diagonal (2022=1.0595) skewing the 3-year window. Given this instability rather than a clean trend, selected near the more stable all-year/10-year trimmed averages (weighted_all=1.3437, avg_exclude_high_low_10yr=1.3658) rather than chasing either extreme window.</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>1.1800 selected. CV_5yr=0.10, CV_3yr=0.050 (low to moderate). 3yr VW=1.133, 5yr VW=1.200, 10yr VW=1.225, all VW=1.180. Moderate divergence between 3yr and 5yr (~5.6%). Recent AYs: 2020=1.121, 2021=1.070, with 2019=1.183 and 2018=1.374. AY2018 (1.374) is notably high (large case reserve emergence). 5yr includes the 2018 spike while 3yr does not. The all-year VW (1.180) falls squarely between 3yr and 5yr and is the most balanced estimate. At mid-early maturity, Bayesian anchoring to the all-year central estimate is appropriate. Selection of 1.180 equals the all-year VW, reflecting a stable central tendency that is consistent with the 10yr VW (1.225) discounted slightly for the likelihood that 2018 was an outlier AY.</t>
+          <t>1.1450: cv_5yr=0.10 triggers single high/low exclusion (avg_exclude_high_low_5yr=1.1437). 3yr (1.1327) sits below 5yr (1.1999), an 5.6% divergence, but lacks clear diagnostic confirmation (no matching severity or closure-rate signal at this maturity), so treated with skepticism per the no-diagnostic-support rule and selected near the outlier-trimmed 5-year average rather than fully weighting the 3-year window.</t>
         </is>
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>1.0800 selected. CV_5yr=0.076 (moderate). 3yr VW=1.108, 5yr VW=1.098, 10yr VW=1.087, all VW=1.104. Recent AYs: 2020=1.011, 2019=1.231, 2018=1.058 — the 3yr is partially elevated by 2019's high factor. The 5yr and 10yr converge near 1.087-1.098. All-year VW = 1.104. Slope over 3yr is negative (-0.024) suggesting recent softening. Selection of 1.080 is slightly below the converging 5yr/10yr range, reflecting the recent declining trend in this column (2020: 1.011) while recognizing that 2020 may be partially COVID-suppressed. The all-year at 1.104 provides an upper bound; the 3yr at 1.108 is modestly inflated by the 2019 spike.</t>
+          <t>1.1000: Convergence Override applies - weighted_all (1.1038), simple_all (1.1009), weighted_5yr (1.0978), weighted_3yr (1.1082) are all within a ~1.4% band. Selected the midpoint of the converged band.</t>
         </is>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
-          <t>1.1100 selected. CV_5yr=0.052, CV_3yr=0.072 (low). 3yr VW=1.129, 5yr VW=1.119, 10yr VW=1.086, all VW=1.077. 3yr and 5yr converge tightly (within 0.9%), both materially above the 10yr (gap ~3.3%). This constitutes partial convergence of the recent windows. The 3yr/5yr convergence at 1.12-1.13 suggests a level shift upward in recent paid development at 59-71 months, consistent with rising incurred severity in recent AYs. Incurred severity at age 59 in 2019 was ~5927, 2018 ~7067 — confirming elevated loss environment. Convergence override of the 3yr/5yr midpoint (1.124) applies; partial discount toward 5yr VW for conservatism yields 1.110.</t>
+          <t>1.1250: 3yr (1.1286) and 5yr (1.1192) weighted averages closely agree and both exceed the all-year average (1.0774) by 4.5%, a diagnostic-confirmed upward trend (rising paid severity in recent accident years). Blended 60% 3yr / 40% 5yr per the 3-5% divergence band, landing at 1.1252, rounded to 1.1250.</t>
         </is>
       </c>
       <c r="G70" s="20" t="inlineStr">
         <is>
-          <t>1.1150 selected. CV_5yr=0.096, CV_3yr=0.101 (moderate). 3yr VW=1.130, 5yr VW=1.107, 10yr VW=1.085, all VW=1.059. Notable upward trend in recent years: 2019 not yet visible at 71-83, 2018: 1.060, 2017: 1.291, 2016: 1.140. The 3yr is elevated by the 2017 spike (1.291); the 5yr VW (1.107) is more balanced. At mid maturity (71-83 months), paid LDFs should be converging with incurred. The corresponding incurred 71-83 selection is 1.075. Paid being higher than incurred here is consistent with the paid-to-incurred ratios still below 1.0 in recent AYs (2019: 0.921, 2018: 0.969 at age 71). Selection of 1.115 is between 5yr VW (1.107) and 3yr VW (1.130), reflecting credible ongoing development. CV&gt;0.10 triggers outlier exclusion consideration — 5yr ex-hi/lo = 1.103 confirms the 5yr VW is reasonable.</t>
+          <t>1.0880: This is a late-maturity column (72+ mo) where recency is normally de-emphasized, but the upward move (weighted_5yr=1.107 vs weighted_all=1.0591, a 4.5% gap) is corroborated cross-view by paid_severity_incr trending up across multiple diagonals, treated as an ongoing inflationary signal (Section 13) rather than a one-time blip. Weighted 60% toward the 5-year average and 40% toward all-year to balance late-maturity caution against the confirmed trend.</t>
         </is>
       </c>
       <c r="H70" s="20" t="inlineStr">
         <is>
-          <t>1.0300 selected. CV_5yr=0.039, CV_3yr=0.040 (low). 3yr VW=1.043, 5yr VW=1.033, 10yr VW=1.026, all VW=1.026. 3yr and 5yr are consistent. All averages converge within ~1.7%, with the 5yr and 10yr/all bracketed around 1.026-1.043. Selection of 1.030 follows the 5yr VW as the primary reference, reflecting stable mid-maturity development. The corresponding incurred 83-95 selection (1.009) being lower than paid (1.030) is consistent with ongoing paid development exceeding incurred at this stage.</t>
+          <t>1.0290: cv_3yr=0.04, cv_5yr=0.04, low variance and reasonable agreement across windows (weighted_all=1.026, weighted_5yr=1.0328, weighted_3yr=1.0426). Selected a value near the all-year/5-year midpoint, consistent with late-maturity preference for the longer window absent a structural break.</t>
         </is>
       </c>
       <c r="I70" s="20" t="inlineStr">
         <is>
-          <t>1.0130 selected. CV_5yr=0.011, CV_3yr=0.004 (very low). All averages converge tightly: 3yr=1.011, 5yr VW=1.013, 10yr VW=1.025, all VW=1.021. The 3yr and 5yr are near-identical (convergence override applies). Selection follows the 5yr VW of 1.013, reflecting stable, low paid development at this late maturity. The 10yr and all-year are slightly higher due to older AYs. No trend signal.</t>
+          <t>1.0170: cv_3yr=0.004 (very low), weighted_all (1.0208), weighted_5yr (1.0132), and weighted_3yr (1.0116) sit within ~1% of each other - effectively converged. Selected the midpoint.</t>
         </is>
       </c>
       <c r="J70" s="20" t="inlineStr">
         <is>
-          <t>1.0550 selected. CV_5yr=0.057, CV_3yr=0.065 (low). 3yr VW=1.098, 5yr VW=1.065, 10yr VW=1.055, all VW=1.039. Recent AYs: 2015 had a very high factor (1.138) and 2014 had 1.062 — the 3yr is elevated by 2015's spike which reflects large case reserve emergence visible in the diagnostics (2015 case reserves at age 107 = 129K). 5yr and 10yr converge around 1.055-1.065. All-year at 1.039 may be slightly low due to older well-reserved AYs. Selection of 1.055 follows the 10yr VW as a balanced estimate that discounts the 2015 spike while staying above the all-year.</t>
+          <t>1.0450: Late-maturity column with few contributing accident years at this depth (sparse-data caution applies). weighted_3yr (1.0982) is notably above weighted_all (1.0394), largely reflecting a single high recent diagonal (2015=1.1378) rather than a broad-based trend. Anchored primarily to the all-year average with a modest upward nudge rather than following the thin recent window.</t>
         </is>
       </c>
       <c r="K70" s="20" t="inlineStr">
         <is>
-          <t>1.0100 selected. CV_5yr=0.012, CV_3yr=0.015 (very low). All averages converge tightly: 3yr=1.012, 5yr VW=1.008, 10yr VW=1.035, all VW=1.028. The 3yr and 5yr converge at 1.008-1.012. The 10yr and all-year are higher due to older AYs with more material development. Selection of 1.010 follows the midpoint of 3yr and 5yr convergence zone, reflecting stable low development at this maturity. AY2015's factor at 119-131 is not yet visible but prior factors support this range.</t>
+          <t>1.0200: weighted_all (1.0282) sits above weighted_5yr (1.0083) and weighted_3yr (1.0133) - the elevated all-year figure reflects older-year spikes (e.g. 2007=1.05, 2012=1.0565) not repeated recently. Blended toward the more current, lower-variance recent windows, cv_5yr=0.012 (low).</t>
         </is>
       </c>
       <c r="L70" s="20" t="inlineStr">
         <is>
-          <t>1.0100 selected. CV_5yr=0.024 (low). 3yr=1.022, 5yr VW=1.019, 10yr VW=1.025, all VW=1.023. All averages converge tightly within 0.6pp. Convergence override applies — select midpoint of converged band (~1.021). Slight downward adjustment to 1.010 for the observation that the most recent AYs with data at this maturity (2013: 1.000, 2012: 1.057, 2011: 1.010) show declining development. The 5yr ex-hi/lo = 1.014 confirms the moderate level.</t>
+          <t>1.0210: Converged across windows - weighted_all (1.0226), weighted_5yr (1.0189), weighted_3yr (1.022) all within ~0.4%. Selected the midpoint; cv_5yr=0.024 confirms low volatility at this depth.</t>
         </is>
       </c>
       <c r="M70" s="20" t="inlineStr">
         <is>
-          <t>1.0150 selected. CV_5yr=0.024 (low). 3yr=1.016, 5yr VW=1.018, 10yr VW=1.022, all VW=1.021. Near-full convergence across all windows (within 0.6pp). Convergence override applies: select midpoint of converged band = 1.015-1.022. Selection of 1.015 reflects the lower end of the convergence zone consistent with the recent 3yr average, which has the most recent information.</t>
+          <t>1.0180: weighted_all (1.0211), weighted_5yr (1.0175), weighted_3yr (1.0138) show a mild downward drift toward recent years, consistent with normal decay at this maturity. Selected between the all-year and 5-year averages.</t>
         </is>
       </c>
       <c r="N70" s="20" t="inlineStr">
         <is>
-          <t>1.0100 selected. CV very low (3yr=0.002, 5yr=0.012). All averages converge: 3yr=1.001, 5yr VW=1.013, 10yr VW=1.010, all VW=1.015. The 10yr and all-year converge at 1.010-1.015. The 3yr is near-zero reflecting recent zero-development AYs. Selection at 1.010 follows the 10yr VW, which best captures the central long-run development level at this mature age, acknowledging that near-term zero factors may understate long-run tail.</t>
+          <t>1.0080: weighted_3yr (1.0016) is markedly lower than weighted_5yr (1.0134) and weighted_all (1.0151), consistent with the expected flattening of development toward 1.0 at this deep maturity (&gt;150 months). Selected between the 3-year and 5-year figures, giving weight to the natural decay pattern rather than the noisier all-year mean.</t>
         </is>
       </c>
       <c r="O70" s="20" t="inlineStr">
         <is>
-          <t>1.0075 selected. CV_5yr=0.011 (very low). All averages converge tightly: 3yr=1.002, 5yr VW=1.014, 10yr VW=1.016, all VW=1.016. The 5yr/10yr/all converge around 1.014-1.016. The 3yr is lower due to recent zero-development AYs. Selection of 1.0075 is below the 5yr to reflect recent declining activity while acknowledging the structural development in the all-year average.</t>
+          <t>1.0090: Same flattening pattern as the prior column - weighted_3yr (1.0023) well below weighted_all (1.0156)/weighted_5yr (1.0143). Selected a value between the recent and longer-term averages, consistent with continued monotonic decay toward unity.</t>
         </is>
       </c>
       <c r="P70" s="20" t="inlineStr">
         <is>
-          <t>1.0025 selected. CV very low. All averages near 1.000-1.020. 3yr=1.019, 5yr VW=1.016, 10yr VW=1.016, all VW=1.016. Most recent AYs showing 1.000 factors. Selection of 1.003 reflects modest residual development, acknowledging that several recent AYs have reached finality at this maturity while older AYs showed more development.</t>
+          <t>1.0170: weighted_all (1.0163), weighted_5yr (1.0156), weighted_3yr (1.0193) are tightly converged (within 0.3%). Selected the midpoint.</t>
         </is>
       </c>
       <c r="Q70" s="20" t="inlineStr">
         <is>
-          <t>[CUTOFF] CUTOFF at 191 months: is_monotone_from_here=True for paid loss. CV at 191+ months is near-zero throughout (3yr=0.010, 5yr=0.010). Factors are stable at 1.000-1.010 range with only a few observations per column. Fewer than 5 credible data points remain in each interval beyond 191 months. Paid loss minimum cutoff is 60 months — this is well exceeded at 191 months. Tail curve fitting commences from 191 months. The sparse data caution (fewer observations per column increasing, near-zero development) combined with the convergence of all averages to 1.000 confirms this as the appropriate cutoff.</t>
-        </is>
-      </c>
-      <c r="R70" s="8" t="n"/>
+          <t>1.0130: weighted_all (1.0158), weighted_5yr (1.0115), weighted_3yr (1.0109) are closely aligned; selected between the all-year and recency-weighted figures. This is the last interval selected before the tail cutoff - cv_5yr=0.0103, low and stable, supporting a credible endpoint for observed development.</t>
+        </is>
+      </c>
+      <c r="R70" s="20" t="inlineStr">
+        <is>
+          <t>[CUTOFF] CUTOFF at 215 months (well beyond the 60-month Paid Loss minimum). From this point on, cv_5yr values are extremely low (0.0031-0.0069, all &lt;0.01) and factors hover in a tight ±1.5% band around 1.0 (1.0021-1.0087) with residual noise-level slope-sign changes rather than a structural break. 7 intervals remain (203-215 through 275-287) for tail curve fitting, comfortably meeting the ≥3-5 requirement. The final column (275-287) has only a single accident-year observation (2001) and cv is undefined, confirming this region is better handled by curve extrapolation than by hand-selection.</t>
+        </is>
+      </c>
       <c r="S70" s="8" t="n"/>
       <c r="T70" s="8" t="n"/>
       <c r="U70" s="8" t="n"/>
@@ -8160,67 +8172,67 @@
         </is>
       </c>
       <c r="B72" s="22" t="n">
-        <v>2.55</v>
+        <v>2.48</v>
       </c>
       <c r="C72" s="22" t="n">
-        <v>1.38</v>
+        <v>1.35</v>
       </c>
       <c r="D72" s="22" t="n">
-        <v>1.18</v>
+        <v>1.185</v>
       </c>
       <c r="E72" s="22" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="F72" s="22" t="n">
-        <v>1.11</v>
+        <v>1.095</v>
       </c>
       <c r="G72" s="22" t="n">
-        <v>1.11</v>
+        <v>1.075</v>
       </c>
       <c r="H72" s="22" t="n">
-        <v>1.035</v>
+        <v>1.028</v>
       </c>
       <c r="I72" s="22" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="J72" s="22" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="K72" s="22" t="n">
         <v>1.02</v>
       </c>
-      <c r="J72" s="22" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="K72" s="22" t="n">
-        <v>1.025</v>
-      </c>
       <c r="L72" s="22" t="n">
-        <v>1.02</v>
+        <v>1.022</v>
       </c>
       <c r="M72" s="22" t="n">
-        <v>1.02</v>
+        <v>1.018</v>
       </c>
       <c r="N72" s="22" t="n">
-        <v>1.01</v>
+        <v>1.012</v>
       </c>
       <c r="O72" s="22" t="n">
-        <v>1.01</v>
+        <v>1.013</v>
       </c>
       <c r="P72" s="22" t="n">
-        <v>1.01</v>
+        <v>1.016</v>
       </c>
       <c r="Q72" s="22" t="n">
-        <v>1.015</v>
+        <v>1.013</v>
       </c>
       <c r="R72" s="22" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="S72" s="22" t="n">
         <v>1.008</v>
       </c>
-      <c r="S72" s="22" t="n">
-        <v>1.01</v>
-      </c>
       <c r="T72" s="22" t="n">
-        <v>1.002</v>
+        <v>1.003</v>
       </c>
       <c r="U72" s="22" t="n">
         <v>1.005</v>
       </c>
       <c r="V72" s="22" t="n">
-        <v>1.007</v>
+        <v>1.006</v>
       </c>
       <c r="W72" s="22" t="n">
         <v>1.007</v>
@@ -8235,117 +8247,117 @@
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>2.5500. The paid loss 11-23 factor is substantially higher than incurred, reflecting slow initial payment. The weighted-all average is 2.457 and simple-all is 2.498. The 3-year average (2.564) and 5-year (2.584) are elevated, driven by years like 2016 (3.315), 2023 (3.265), 2009 (3.246). The 10-year weighted average is 2.482. The paid-to-incurred ratio at 11 months averages around 40-70%, confirming significant unpaid at initial evaluation. Recent years show a wide range: 2022 (2.429), 2021 (1.998), 2020 (2.554), 2019 (2.675), 2018 (2.875), 2017 (1.737). The low 2017 and 2021 factors stand out as outliers. CV is moderate at 0.23 for the 10-year window. A selection of 2.55 is slightly above the weighted-all (2.457) and near the exclude-high-low-all average (2.495), reflecting the upward trend in recent years relative to historical and the generally elevated recent factors.</t>
+          <t>2.48 selected. This is the largest and most volatile link in the paid triangle (cv_3yr 0.25) reflecting early-duration claim payment ramp-up. Individual factors range from 1.74 (2017) to 3.32 (2016) with no clear directional trend across origin years, so a long-window average is more credible than a short one. The value sits between weighted_all (2.4566) and weighted_10yr (2.482), essentially the 10-year weighted average, which balances the high recent years (2018: 2.8751, 2023: 3.2653) against lower ones (2020: 2.5535, 2021: 1.9981) without overweighting any single cohort.</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>1.3800. The weighted-all is 1.344 and simple-all is 1.339. The 5-year averages are around 1.428 and the 3-year is around 1.302 (weighted). The paid development at this age remains substantial — paid-to-incurred at 23 months is still in the 60-93% range for most years. Recent years show high factors: 2019 (1.750), 2018 (1.484), 2021 (1.666). The 5-year simple average of 1.428 is elevated relative to the long-run average of 1.339. CV is high at 0.19-0.21, indicating meaningful variability. A selection of 1.38 is between the all-period weighted (1.344) and the 5-year (1.428), giving partial weight to the recent uptick in development while not fully crediting the most recent 3 years which include unusually high values.</t>
+          <t>1.35 selected, close to weighted_10yr (1.3913) and simple_all (1.3387). CV is still elevated (0.25 at 3yr) with individual factors from 1.06 (2022) to 1.75 (2019). Recent 3-year weighted (1.2671) is somewhat lower, but given the volatility and no consistent trend, a full-history-anchored value is preferred over over-fitting to 3 recent points.</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>1.1800. The weighted-all is 1.180 and simple-all is 1.172. The 3-year average is 1.124 and 5-year is 1.200. The 10-year weighted is 1.225. Notable outliers include 2015 (1.465), 2008 (1.367), 2001 (1.236). Recent years 2020 (1.121), 2021 (1.070), 2022 (N/A) are lower. CV is 0.10-0.11, indicating reasonable stability in the middle of the range. The paid-to-incurred ratio at 35 months ranges from 70-99%, suggesting most but not all development has occurred. A selection of 1.18 aligns with the weighted-all average, balanced across time periods.</t>
+          <t>1.185 selected. Development moderates meaningfully here; averages cluster tightly (weighted_all 1.1803, 5yr 1.1999, 10yr 1.2249, 3yr 1.1327) with cv_3yr only 0.05 — good stability. Selection sits near the middle of the recent windows, slightly below the longer-term averages given the softer 3-year figure.</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>1.0900. The weighted-all is 1.104 and simple-all is 1.101. The 3-year simple average is 1.100. The 5-year averages range 1.087-1.092. Recent years: 2019 (1.231), 2020 (1.011), 2021 (N/A). The 2019 factor is an outlier. CV is 0.064-0.076. A selection of 1.09 is slightly below the all-period weighted (1.104) but acknowledges the volatile recent experience and reflects the majority of mid-period years which cluster in the 1.05-1.19 range.</t>
+          <t>1.10 selected. Averages agree closely across windows (weighted_all 1.1038, 3yr 1.1082, 5yr 1.0978, 10yr 1.0874), indicating a stable, credible pattern with low dispersion. Selection is essentially the consensus of all four averages.</t>
         </is>
       </c>
       <c r="F73" s="24" t="inlineStr">
         <is>
-          <t>1.1100. The weighted-all is 1.077 and simple-all is 1.067, but the recent 3-year and 5-year averages are materially higher at 1.119-1.129. Recent years show a distinct uptick: 2017 (1.108), 2018 (1.056), 2019 (1.215). This interval has been systematically elevated in the most recent 5 accident years visible in the data, consistent with the slow payment trend in recent years. CV is 0.052-0.063. A selection of 1.11 weights the recent 5-year experience (1.119) more heavily than the long-run average (1.077) to reflect the apparent shift in payment pace.</t>
+          <t>1.095 selected. Recent years run modestly above the all-year average (weighted_3yr 1.1286, 5yr 1.1192 vs weighted_all 1.0774), suggesting slightly more late development recently (e.g., 2019: 1.2153). Selection leans toward the recent windows while not fully abandoning the longer history.</t>
         </is>
       </c>
       <c r="G73" s="24" t="inlineStr">
         <is>
-          <t>1.1100. The weighted-all is 1.059 and simple-all is 1.056, but the 3-year average is 1.164 and 5-year is 1.107-1.122. Recent high factors: 2017 (1.291), 2016 (1.140), 2015 (1.111). The 2017 factor of 1.291 is a significant outlier. Even excluding that, recent development has run well above the long-run average. CV is 0.082-0.097, indicating meaningful dispersion. A selection of 1.11 reflects the 5-year weighted average (1.107) and acknowledges the elevated recent development, while the 2017 outlier keeps the 3-year average from being fully credible.</t>
+          <t>1.075 selected, near weighted_10yr (1.0846) and between weighted_all (1.0591) and the elevated 3yr/5yr figures (1.13, 1.107) that are influenced by a large 2017 factor (1.2914). Moderating the recent-year spike with longer history avoids overreacting to one outlier year.</t>
         </is>
       </c>
       <c r="H73" s="24" t="inlineStr">
         <is>
-          <t>1.0350. The weighted-all is 1.026 and simple-all is 1.023. The 3-year simple average is 1.051 and 5-year is 1.031. Notable factors include 2009 (1.050) and 2017 (1.091). CV is 0.031-0.039. Most years are in the 1.000-1.080 range. A selection of 1.035 is above the all-period average to reflect recent elevated experience and the upward shift in this interval in recent periods.</t>
+          <t>1.028 selected, consistent with weighted_all (1.026), 10yr (1.0256) and simple_all (1.0233). Development has largely tapered; all windows agree closely, so the selection is a simple consensus value.</t>
         </is>
       </c>
       <c r="I73" s="24" t="inlineStr">
         <is>
-          <t>1.0200. The weighted-all is 1.021, simple-all is 1.018. The 3-year is 1.011 and 5-year is 1.013. The 2007 factor (1.081) and 2009 (1.037) are higher outliers. CV is moderate (0.024-0.024). Most years are in 1.000-1.082 range. A selection of 1.020 aligns with the weighted-all average.</t>
+          <t>1.018 selected, between weighted_all (1.0208) and the milder recent windows (3yr 1.0116, 5yr 1.0132). Tail development continues to shrink with maturity; selection reflects a gentle blend favoring recent experience slightly.</t>
         </is>
       </c>
       <c r="J73" s="24" t="inlineStr">
         <is>
-          <t>1.0400. The weighted-all is 1.039 and simple-all is 1.028. The 3-year simple average is 1.067 and 5-year is 1.064. Notable outliers: 2015 (1.138), 2007 (1.085). Recent years show elevated development. CV is 0.044-0.057. A selection of 1.040 reflects the weighted-all average, acknowledging continued development at this age.</t>
+          <t>1.045 selected. This interval shows elevated volatility (cv_3yr 0.0647) driven by a few years with meaningful late reopenings/payments (2015: 1.1378, 2011: 1.0922), pulling the 3-year weighted average up to 1.0982. Selection splits the difference between the long-run average (1.0394) and the higher recent signal, acknowledging some real upward development risk without fully adopting the spike.</t>
         </is>
       </c>
       <c r="K73" s="24" t="inlineStr">
         <is>
-          <t>1.0250. The weighted-all is 1.028 and simple-all is 1.022. The 3-year simple is 1.012 and 5-year is 1.009. Some years show notable development: 2006 (1.092), 2007 (1.082), 2015 (N/A). CV is 0.033 for 10-year. A selection of 1.025 is between the recent low averages and the all-period weighted, reflecting residual development.</t>
+          <t>1.020 selected, close to weighted_all (1.0282) and simple_all (1.0221), moderating the high 10yr figure (1.0353) which is influenced by a couple of larger factors (2012: 1.0297, 2016 n/a). Reasonable central estimate for a maturing but still slowly developing interval.</t>
         </is>
       </c>
       <c r="L73" s="24" t="inlineStr">
         <is>
-          <t>1.0200. Weighted-all is 1.023 and simple-all is 1.019. The 3-year is 1.022 and 5-year is 1.020. CV is low at 0.020-0.024. A selection of 1.020 is consistent with both the all-period and recent averages.</t>
+          <t>1.022 selected, consistent with weighted_all (1.0226), 3yr (1.022) and 5yr (1.0189). Factors are broadly stable in the low single-digit-percent range at this maturity.</t>
         </is>
       </c>
       <c r="M73" s="24" t="inlineStr">
         <is>
-          <t>1.0200. Weighted-all is 1.021, simple-all is 1.019. The 3-year and 5-year averages are 1.014-1.020. CV is low (0.020-0.024). A selection of 1.020 reflects the pattern well.</t>
+          <t>1.018 selected, between weighted_all (1.0211) and the somewhat lower recent 3yr figure (1.0138). Consistent, modest late development continues.</t>
         </is>
       </c>
       <c r="N73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.015, simple-all is 1.011. The 5-year is 1.013 and 3-year is 1.001. Factors range 1.000-1.029. CV is 0.012. A selection of 1.010 reflects the all-period central tendency.</t>
+          <t>1.012 selected, close to weighted_all (1.0151) and 10yr (1.0137), slightly tempered toward the very low 3yr figure (1.0016) which reflects a run of near-unity recent factors.</t>
         </is>
       </c>
       <c r="O73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.016, simple-all is 1.011. CV is low. Factors mostly in 1.000-1.030 range. A selection of 1.010 is appropriate.</t>
+          <t>1.013 selected, near weighted_all (1.0156) and 10yr (1.0156). Development is small and fairly consistent across origin years at this maturity.</t>
         </is>
       </c>
       <c r="P73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.016, simple-all is 1.012. The 5-year is 1.010 and 3-year is 1.011. CV is 0.012-0.016. Modest but consistent development. A selection of 1.010 aligns with both the recent and all-period averages.</t>
+          <t>1.016 selected, matching weighted_all (1.0163) and 10yr (1.0163) closely; recent years show similar levels (3yr 1.0193).</t>
         </is>
       </c>
       <c r="Q73" s="24" t="inlineStr">
         <is>
-          <t>1.0150. Weighted-all is 1.016, simple-all is 1.016. The 5-year average is 1.013. CV is low. The 2001 factor (1.033) and 2008 (1.026) are higher outliers. A selection of 1.015 aligns with the all-period averages.</t>
+          <t>1.013 selected, between weighted_all (1.0158) and the lower recent windows (3yr 1.0109, 5yr 1.0115). Development continues to gently decay with maturity.</t>
         </is>
       </c>
       <c r="R73" s="24" t="inlineStr">
         <is>
-          <t>1.0080. Weighted-all is 1.009 and simple-all is 1.008. CV is very low. Most factors at or near 1.000. A selection of 1.008 is consistent with the all-period average.</t>
+          <t>1.006 selected, consistent with weighted_all (1.0087) and 10yr (1.0087), moderated slightly toward the very low 3yr/5yr figures (~1.003).</t>
         </is>
       </c>
       <c r="S73" s="24" t="inlineStr">
         <is>
-          <t>1.0100. Weighted-all is 1.013 and simple-all is 1.010. Some development continues — 2001 (1.038), 2002 (1.016). CV is 0.015. A selection of 1.010 reflects the simple-all average.</t>
+          <t>1.008 selected, near weighted_all (1.013) and 10yr (1.013); this interval is influenced by one larger factor (2001: 1.0383) against several near-unity years, so the selection sits below the mean-driven averages to avoid overweighting the single outlier.</t>
         </is>
       </c>
       <c r="T73" s="24" t="inlineStr">
         <is>
-          <t>1.0020. Weighted-all and simple-all are both 1.002-1.002. Only a few observations (2001: 1.000, 2002: 1.012). Very sparse. A selection of 1.002 is minimal, reflecting near-flat development at this age.</t>
+          <t>1.003 selected, consistent with weighted_all (1.0025) and 5yr/10yr (1.0025). Development is now very minor and highly consistent.</t>
         </is>
       </c>
       <c r="U73" s="24" t="inlineStr">
         <is>
-          <t>1.0050. Weighted-all is 1.005, simple-all is 1.004. Observations: 2001 (1.007), 2002 (1.010). CV is very low. A selection of 1.005 is consistent.</t>
+          <t>1.005 selected, matching weighted_all, 5yr, and 10yr averages (all 1.0054). Small, stable residual development.</t>
         </is>
       </c>
       <c r="V73" s="24" t="inlineStr">
         <is>
-          <t>1.0070. Weighted-all and simple-all are 1.006-1.008. Observations: 2001 (1.007), 2002 (1.010). A selection of 1.007 is consistent with observed values.</t>
+          <t>1.006 selected, matching weighted_all and other windows (all ~1.0062). Consistent minor tail development.</t>
         </is>
       </c>
       <c r="W73" s="24" t="inlineStr">
         <is>
-          <t>1.0070. Only one observation at 263-275 (2001: 1.006) and one at 275-287 (2001: 1.004). The weighted/simple-all averages are 1.007-1.008. A selection of 1.007 uses the available averages.</t>
+          <t>1.007 selected, matching the only two data points available (2001: 1.0063, 2002: 1.009) which are tightly clustered, giving reasonable confidence despite thin volume. This is the last interval selected directly from data before volume becomes too sparse for a credible standalone factor.</t>
         </is>
       </c>
       <c r="X73" s="24" t="inlineStr">
         <is>
-          <t>[CUTOFF] Cutoff at 275 months. Only a single observation is available (2001: 1.004), making any direct selection unreliable. At 275+ months the data is exhausted and a tail curve should take over. The tail factor from 275 months to ultimate should be estimated using an actuarial decay curve fitted to the 191-275 interval pattern.</t>
+          <t>[CUTOFF] Cutoff at 287: only a single origin year (2001) has data at this maturity, providing no cross-sectional credibility to validate a factor. Beyond this point, a fitted tail curve (e.g., inverse power or exponential decay) is more reliable than a one-observation direct selection for extrapolating the remaining runout.</t>
         </is>
       </c>
     </row>
@@ -11932,17 +11944,17 @@
     <row r="69">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Selection</t>
+          <t>Framework AI Selection</t>
         </is>
       </c>
       <c r="B69" s="18" t="n">
-        <v>1.09</v>
+        <v>1.118</v>
       </c>
       <c r="C69" s="18" t="n">
-        <v>1.002</v>
+        <v>1.001</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>1</v>
+        <v>1.0005</v>
       </c>
       <c r="E69" s="18" t="n">
         <v>1</v>
@@ -11972,37 +11984,37 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="17" t="inlineStr">
         <is>
-          <t>Rules-Based AI Reasoning</t>
+          <t>Framework AI Reasoning</t>
         </is>
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>1.0900 selected. CV_5yr=0.032, CV_3yr=0.013 (very low). All averages are well-defined and internally consistent: 3yr VW=1.133, 5yr VW=1.118, 10yr VW=1.096, all VW=1.062. A notable upward trend exists in the 11-23 column over recent years: 2017=1.124, 2018=1.123, 2019=1.143, 2020=1.060, 2021=1.142, 2022=1.141, 2023=1.116. The 3yr slope is negative (-0.013) and 5yr slope is positive (+0.003), suggesting the very recent AY2023 pulled the 3yr down from the plateau around 1.12-1.14 reached in 2017-2022. The 5yr VW (1.118) captures the sustained elevated period well. The 10yr VW (1.096) includes earlier lower-reporting years (2008-2010 were around 1.047-1.064). The all-year (1.062) is dragged down by 2011's 1.000, which appears anomalous (no new claims reported between 11 and 23 months for 2011). The 5yr/3yr divergence is ~1.5%, within the 3% Bayesian anchoring threshold — no regime change required. AY2023 at 1.116 confirms the factor remains in the 1.10-1.14 band. Selection of 1.090 reflects a modest conservatism below the 5yr VW (1.118), acknowledging the recent slight softening in 2023 (1.116) and 2020 (1.060 — potential COVID-related reporting delay). This is approximately midpoint of the 10yr VW (1.096) and 5yr VW (1.118).</t>
+          <t>1.1180: Selected the 5-year volume-weighted average. cv_5yr=0.032 is low (good credibility), and weighted_3yr (1.133) and weighted_5yr (1.118) agree closely (1.3% apart, below the 3% divergence threshold that would trigger a 3-year override), both clearly above the all-year average (1.0617). Individual factors show a gradual increase from the early 2000s (~1.03-1.07) to recent years (~1.11-1.14), a genuine, sustained shift toward faster early reporting rather than a one-off spike - supported by using the recency-weighted rather than all-year figure.</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
         <is>
-          <t>1.0020 selected. CV_5yr=0.000, CV_3yr=0.000 (essentially zero). All averages across every window are 1.000 or 1.001-1.008: 3yr=1.000, 5yr=1.000, 10yr VW=1.007, all VW=1.003. Only 2 AYs show non-1.000 factors: 2001 (1.002), 2009 (1.004), 2014 (1.003), 2015 (1.016), 2016 (1.046). The 2016 factor of 1.046 is a clear outlier (most likely a small administrative re-opening of claims). Nearly all AYs in the last decade show exactly 1.000. The 10yr VW is 1.007 — driven by the 2016 outlier. Selection of 1.002 follows the all-year VW, acknowledging that very occasionally a small number of late-reported claims arrive between 23 and 35 months but the pattern is near-zero. Convergence override applies (all windows within 1.6% of each other with near-zero CV).</t>
+          <t>1.0010: Convergence Override - weighted_all (1.0033), simple_all (1.0037), weighted_5yr (1.0), weighted_3yr (1.0), and avg_exclude_high_low_all (1.0018) are all within a very tight band (&lt;0.4% spread), with cv values near zero across all windows. Selected the midpoint of the converged band.</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>1.0000 selected. CV_5yr=0.002 (essentially zero). All averages converge tightly at 1.000: 3yr=1.000, 5yr=1.001, 10yr=1.001, all VW=1.000. The only non-1.000 factors in the triangle are 2001 (1.000 — barely rounds), 2004 (1.004), 2009 (1.000), 2013 (1.005). These are trivially small. Reported counts are fully developed by 35 months in virtually all AYs. Convergence override applies — full convergence to 1.000. Select 1.000.</t>
+          <t>1.0005: Convergence Override - all averaging windows sit between 1.0 and 1.0009 (weighted_all=1.0004, weighted_5yr=1.0008, weighted_3yr=1.0), cv near zero. Selected the midpoint, reflecting the near-complete reporting of claim counts by this maturity.</t>
         </is>
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>1.0000 selected. CV_5yr=0.003 (essentially zero). All averages: 3yr=1.001, 5yr=1.000, all VW=1.000. Only minor non-1.000 factors in a handful of AYs (e.g., 2004: 1.002, 2013: 1.000, 2018: 1.004, 2017: 0.996). Both positive and negative deviations of &lt;0.5%. Fully converged — select 1.000.</t>
+          <t>1.0000: Convergence Override - weighted_all (0.9998), weighted_5yr (1.0), weighted_3yr (1.0013) are all essentially at unity with near-zero CV. Reported counts are effectively fully developed by this maturity; selected 1.0000, consistent with reported-count development never needing a sub-1.000 factor at this stage absent claim count restatements (none observed in the diagnostics).</t>
         </is>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
-          <t>1.0000 selected. CV_5yr=0.002 (essentially zero). All averages at 0.999-1.002. Tiny deviations only. No systematic development beyond 47 months in reported counts. Select 1.000 — full convergence.</t>
+          <t>1.0000: All averaging windows converge at or just below/above unity (weighted_all=1.0019, weighted_5yr=0.9992, weighted_3yr=0.9987) with cv effectively zero. Selected 1.0000 as the stable, fully-converged reading; this is the last interval selected before the tail cutoff.</t>
         </is>
       </c>
       <c r="G70" s="20" t="inlineStr">
         <is>
-          <t>[CUTOFF] CUTOFF at 71 months: is_monotone_from_here=True. CV is 0.000 for all windows at 71+ months. All factors are 1.000 for virtually every AY from 71 months onward (with only trivial exceptions at earlier intervals). No credible or material development exists beyond 71 months for reported counts. Minimum cutoff for Reported Count is 48 months — this is exceeded. Tail factor for reported count should be 1.000 from 71 months onward. There are 5 intervals remaining (71-83 through 275-287) for tail curve fit, all of which will be 1.000.</t>
+          <t>[CUTOFF] CUTOFF at 83 months (comfortably beyond the 48-month Reported Count minimum). From 71-83 onward, factors are at or extremely close to 1.0 across every averaging window (cv_5yr=0.0 for nearly every remaining column) with no monotonic-decay concerns since there is essentially nothing left to develop - reported claim counts are fully emerged by this point in the data. 17 intervals remain (71-83 through 263-275) for tail curve fitting, far exceeding the ≥3-5 requirement. No structural breaks or diagnostic signals (claim closure, reopenings) suggest any further count development is needed beyond this point.</t>
         </is>
       </c>
       <c r="H70" s="8" t="n"/>
@@ -12031,13 +12043,13 @@
         </is>
       </c>
       <c r="B72" s="22" t="n">
-        <v>1.07</v>
+        <v>1.09</v>
       </c>
       <c r="C72" s="22" t="n">
-        <v>1.003</v>
+        <v>1.004</v>
       </c>
       <c r="D72" s="22" t="n">
-        <v>1</v>
+        <v>1.001</v>
       </c>
       <c r="E72" s="22" t="n">
         <v>1</v>
@@ -12063,16 +12075,36 @@
       <c r="L72" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="M72" s="23" t="n"/>
-      <c r="N72" s="23" t="n"/>
-      <c r="O72" s="23" t="n"/>
-      <c r="P72" s="23" t="n"/>
-      <c r="Q72" s="23" t="n"/>
-      <c r="R72" s="23" t="n"/>
-      <c r="S72" s="23" t="n"/>
-      <c r="T72" s="23" t="n"/>
-      <c r="U72" s="23" t="n"/>
-      <c r="V72" s="23" t="n"/>
+      <c r="M72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="R72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="T72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U72" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="V72" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="W72" s="23" t="n"/>
       <c r="X72" s="23" t="n"/>
     </row>
@@ -12084,74 +12116,114 @@
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>1.0700. Reported count development is highly concentrated at 11-23, with virtually no development thereafter. The weighted-all average is 1.062 and simple-all is 1.068. The 3-year average is 1.133 (simple), reflecting recent elevated reporting: 2022 (1.141), 2021 (1.142), 2023 (1.116), 2017 (1.124), 2018 (1.123), 2019 (1.143). There is a visible upward shift in recent years — 2017-2023 all show factors of 1.10-1.14, markedly above the 2001-2010 range of 1.03-1.07. The 5-year average is 1.118-1.120. This suggests a genuine shift in reporting patterns in more recent accident years toward more late emergence. However, the most recent years (2021, 2022) may partly reflect IBNR patterns that are maturing. A selection of 1.070 is intentionally conservative — it weights the long-run pattern more heavily than the recent 5 years, acknowledging that some of the recent elevated factors may be cyclical. A higher selection around 1.10 would be defensible if recent-year reporting behavior is expected to persist.</t>
+          <t>1.090 selected. This is essentially a claim-count triangle where nearly all development happens between the first two valuations as late-reported claims come in. Individual factors range from 1.0 (2011) to 1.14 (2019/2021/2022), and the more recent origin years (2017-2023) run consistently higher (avg ~1.11-1.13) than the full 24-year history (weighted_all 1.0617, simple_all 1.0679). Selection leans toward the recent experience (weighted_3yr 1.133, weighted_5yr 1.118) tempered slightly by the longer-term level, reflecting a plausible modest lengthening of reporting patterns in recent years.</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>1.0030. After 23 months, count development is essentially complete. The weighted-all is 1.003, simple-all is 1.004. The 3-year and 5-year averages are 1.000 in all windows. CV is extremely low (0.000-0.015). Only 2016 (1.046) and 2008 (1.004) show any meaningful development at this age. The remaining years are 1.000 or within rounding. A selection of 1.003 captures trace development from the occasional late-reported claim.</t>
+          <t>1.004 selected, matching weighted_all (1.0033) and simple_all (1.0037) closely. A handful of years show minor late reporting (2016: 1.0459, 2015: 1.0159) but the pattern is otherwise flat (1.0) across the vast majority of origin years, so a small allowance above unity is appropriate.</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. Virtually no development beyond 35 months. The weighted-all is 1.000, simple-all is 1.001. The max across all years is 1.005 (2013). CV is essentially zero. Selected at 1.000.</t>
+          <t>1.001 selected. Nearly all origin years show exactly 1.0 at this maturity, with only isolated small factors (2004: 1.0041, 2013: 1.0045, 2017: 1.0042). Reported counts are essentially fully developed by this point.</t>
         </is>
       </c>
       <c r="E73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. Development is negligible. Weighted-all and simple-all are essentially 1.000. Only minor fluctuations (2003: 0.995, 2004: 1.002). CV is 0.000-0.002. Selected at 1.000.</t>
+          <t>1.000 selected. All but two origin years (2003: 0.9952, 2017: 0.9958) show exactly 1.0, reflecting claim count closures/reclassifications that roughly offset late reports. Counts are effectively fully reported by this maturity.</t>
         </is>
       </c>
       <c r="F73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. All averages are 1.000 or within rounding (min observed: 0.996, max: 1.027). Only 2001 (1.025) and 2002 (1.027) show any positive development, likely administrative adjustments. Selected at 1.000.</t>
+          <t>1.000 selected. The pattern is flat at 1.0 across nearly all origin years, with isolated minor exceptions (2002: 1.027, 2019: 0.9963) that net out. No further meaningful reported-count development is expected.</t>
         </is>
       </c>
       <c r="G73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. No meaningful development. All averages are 1.000 or rounding noise. Selected at 1.000.</t>
+          <t>1.000 selected. Flat at 1.0 for all origin years except a single outlier (2001: 1.0251), which reflects a minor reclassification rather than ongoing reporting activity.</t>
         </is>
       </c>
       <c r="H73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. No meaningful development. All averages 1.000. Selected at 1.000.</t>
+          <t>1.000 selected. The pattern is flat at 1.0 across all origin years (one minor exception at 2017: 0.9958). Claim counts are fully reported by this maturity for this book.</t>
         </is>
       </c>
       <c r="I73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. Flat — all factors are exactly 1.000 across all periods. No development whatsoever.</t>
+          <t>1.000 selected. All observed factors equal 1.0 with no exceptions in the data shown. No further count development expected.</t>
         </is>
       </c>
       <c r="J73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. All factors are exactly 1.000 except 2015 (0.988 — a downward adjustment, likely closure). No upward development. Selected at 1.000.</t>
+          <t>1.000 selected. All factors equal 1.0 except a single small downward move (2015: 0.9883), likely a claim reclassification/consolidation rather than genuine late reporting. The flat pattern otherwise fully supports unity.</t>
         </is>
       </c>
       <c r="K73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. All factors are 1.000 across all periods. No development.</t>
+          <t>1.000 selected. All observed factors are exactly 1.0 — counts are fully reported and stable by this maturity.</t>
         </is>
       </c>
       <c r="L73" s="24" t="inlineStr">
         <is>
-          <t>1.0000. All factors are 1.000 across all periods. No development.</t>
+          <t>1.000 selected, consistent with a completely flat pattern (all factors 1.0) at this and later maturities.</t>
         </is>
       </c>
       <c r="M73" s="24" t="inlineStr">
         <is>
-          <t>[CUTOFF] Cutoff at 143 months. From 35 months onward, reported count development is exactly 1.000 with no exceptions beyond rounding. The chain-ladder method adds no value beyond 143 months for this measure. A tail factor of 1.000 is appropriate from this point forward, or the count triangle can be considered fully mature at 35 months with a 1.000 tail.</t>
-        </is>
-      </c>
-      <c r="N73" s="11" t="n"/>
-      <c r="O73" s="11" t="n"/>
-      <c r="P73" s="11" t="n"/>
-      <c r="Q73" s="11" t="n"/>
-      <c r="R73" s="11" t="n"/>
-      <c r="S73" s="11" t="n"/>
-      <c r="T73" s="11" t="n"/>
-      <c r="U73" s="11" t="n"/>
-      <c r="V73" s="11" t="n"/>
-      <c r="W73" s="11" t="n"/>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="N73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="O73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="P73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="Q73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="R73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="S73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="T73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="U73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development.</t>
+        </is>
+      </c>
+      <c r="V73" s="24" t="inlineStr">
+        <is>
+          <t>1.000 selected. Flat pattern continues with no observed development; this is the last maturity with reasonable cross-sectional support (multiple origin years) in the provided age-to-age data.</t>
+        </is>
+      </c>
+      <c r="W73" s="24" t="inlineStr">
+        <is>
+          <t>[CUTOFF] Cutoff at 275: reported claim counts have been completely flat at 1.000 for over a dozen consecutive intervals and only the oldest origin years (2001-2003) reach this maturity, leaving minimal volume to test. Given the count triangle is fully developed well before this point, a unity/flat tail assumption (rather than a fitted curve or further direct selection) is the appropriate way to close out the remaining maturities.</t>
+        </is>
+      </c>
       <c r="X73" s="11" t="n"/>
     </row>
     <row r="74"/>

</xml_diff>